<commit_message>
docs: level 1 sign off
</commit_message>
<xml_diff>
--- a/apps/cav-align/governance/Governance_Matrix.xlsx
+++ b/apps/cav-align/governance/Governance_Matrix.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="76">
   <si>
     <t>Release Date</t>
   </si>
@@ -240,9 +240,6 @@
   </si>
   <si>
     <t>alignment_sessions rows created on start/stop</t>
-  </si>
-  <si>
-    <t>M</t>
   </si>
   <si>
     <t>Hardening Complete</t>
@@ -686,7 +683,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -771,15 +768,10 @@
         <v>20</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="B4" t="s">
-        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>